<commit_message>
更新 Telegram 獎品網址整理 2026-03-23 18:40
</commit_message>
<xml_diff>
--- a/Yahoo獎項網址彙整.xlsx
+++ b/Yahoo獎項網址彙整.xlsx
@@ -466,7 +466,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.300000000000001" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="24.1" customWidth="1" min="2" max="2"/>
     <col width="35.1" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
@@ -1119,7 +1119,11 @@
       <c r="A18" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -1156,7 +1160,11 @@
       <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="inlineStr"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -1193,7 +1201,11 @@
       <c r="A20" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -1230,7 +1242,11 @@
       <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="inlineStr"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -1267,7 +1283,11 @@
       <c r="A22" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -1304,7 +1324,11 @@
       <c r="A23" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="inlineStr"/>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
           <t>85度C 58元切片蛋糕</t>
@@ -1341,7 +1365,11 @@
       <c r="A24" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
           <t>85度C 58元切片蛋糕</t>
@@ -1378,7 +1406,11 @@
       <c r="A25" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="inlineStr"/>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
           <t>85度C 58元切片蛋糕</t>
@@ -1415,7 +1447,11 @@
       <c r="A26" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>85度C 58元切片蛋糕</t>
@@ -2224,7 +2260,11 @@
       <c r="A47" s="3" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
           <t>肯德基咔啦脆雞脆薯套餐</t>
@@ -2261,7 +2301,11 @@
       <c r="A48" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
           <t>肯德基咔啦脆雞脆薯套餐</t>
@@ -2298,7 +2342,11 @@
       <c r="A49" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
           <t>肯德基咔啦脆雞脆薯套餐</t>
@@ -42693,7 +42741,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -42708,7 +42756,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -42738,7 +42786,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -43593,7 +43641,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="11.1" customWidth="1" min="2" max="2"/>
     <col width="30.2" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
@@ -43654,7 +43702,11 @@
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -43691,7 +43743,11 @@
       <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -43728,7 +43784,11 @@
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -43765,7 +43825,11 @@
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -43802,7 +43866,11 @@
       <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>蔥花@千</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>摩斯漢堡蛋堡套餐（早餐限定）</t>
@@ -43850,7 +43918,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.2" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="24.1" customWidth="1" min="2" max="2"/>
     <col width="22.6" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
@@ -43911,7 +43979,11 @@
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>85度C 58元切片蛋糕</t>
@@ -43948,7 +44020,11 @@
       <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>85度C 58元切片蛋糕</t>
@@ -43985,7 +44061,11 @@
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>85度C 58元切片蛋糕</t>
@@ -44022,7 +44102,11 @@
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>85度C 58元切片蛋糕</t>
@@ -44914,7 +44998,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.1" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="24.1" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
@@ -44975,7 +45059,11 @@
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>肯德基咔啦脆雞脆薯套餐</t>
@@ -45012,7 +45100,11 @@
       <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>肯德基咔啦脆雞脆薯套餐</t>
@@ -45049,7 +45141,11 @@
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>蝦皮@tobylin60 預留</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>肯德基咔啦脆雞脆薯套餐</t>

</xml_diff>

<commit_message>
更新 Telegram 獎品網址整理 2026-04-16 17:42
</commit_message>
<xml_diff>
--- a/Yahoo獎項網址彙整.xlsx
+++ b/Yahoo獎項網址彙整.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\myhome\Desktop\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44149850-3C09-4D3A-A72C-E6A3DC7058A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0296E526-1962-415C-A140-627EEA88A8CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13126" uniqueCount="2109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13128" uniqueCount="2111">
   <si>
     <t>#</t>
   </si>
@@ -6362,7 +6362,15 @@
     <t>金額合計</t>
   </si>
   <si>
-    <t>千千</t>
+    <t>1150416補era325</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://txp.rs/viewvoucher.aspx?voucherguid=e852122a-337b-4e8e-b2b2-fba2c9afb101</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1150415千千</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -6370,7 +6378,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6388,6 +6396,14 @@
       <name val="新細明體"/>
       <family val="3"/>
       <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="新細明體"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -6423,10 +6439,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -6443,9 +6460,13 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="超連結" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -8168,7 +8189,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>2108</v>
+        <v>2110</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>174</v>
@@ -8194,7 +8215,6 @@
       <c r="A58" s="3">
         <v>57</v>
       </c>
-      <c r="B58" s="4"/>
       <c r="C58" s="3" t="s">
         <v>174</v>
       </c>
@@ -8219,7 +8239,6 @@
       <c r="A59" s="3">
         <v>58</v>
       </c>
-      <c r="B59" s="4"/>
       <c r="C59" s="3" t="s">
         <v>174</v>
       </c>
@@ -8866,7 +8885,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>2108</v>
+        <v>2110</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>242</v>
@@ -8892,15 +8911,17 @@
       <c r="A86" s="3">
         <v>85</v>
       </c>
-      <c r="B86" s="4"/>
+      <c r="B86" s="4" t="s">
+        <v>2108</v>
+      </c>
       <c r="C86" s="3" t="s">
         <v>242</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E86" s="3" t="s">
-        <v>246</v>
+      <c r="E86" s="6" t="s">
+        <v>2109</v>
       </c>
       <c r="F86" s="3"/>
       <c r="G86" s="3" t="s">
@@ -8917,7 +8938,9 @@
       <c r="A87" s="3">
         <v>86</v>
       </c>
-      <c r="B87" s="4"/>
+      <c r="B87" s="4" t="s">
+        <v>2108</v>
+      </c>
       <c r="C87" s="3" t="s">
         <v>242</v>
       </c>
@@ -32879,6 +32902,9 @@
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="E86" r:id="rId1" xr:uid="{EB77AF2F-FF8C-4DB0-A726-2EB08E968FE4}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
更新 Telegram 獎品網址整理 2026-04-22 23:01
</commit_message>
<xml_diff>
--- a/Yahoo獎項網址彙整.xlsx
+++ b/Yahoo獎項網址彙整.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\myhome\Desktop\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44ECE76-FD79-42E4-98ED-66386062E204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08A1CA1-AFE3-4FD6-B3A3-25C94C170D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13280" uniqueCount="2114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13282" uniqueCount="2115">
   <si>
     <t>#</t>
   </si>
@@ -6378,6 +6378,10 @@
   </si>
   <si>
     <t>1150419我</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1150421-tobylin60</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -7859,7 +7863,9 @@
       <c r="A44" s="3">
         <v>43</v>
       </c>
-      <c r="B44" s="4"/>
+      <c r="B44" s="4" t="s">
+        <v>2114</v>
+      </c>
       <c r="C44" s="3" t="s">
         <v>133</v>
       </c>
@@ -7884,7 +7890,9 @@
       <c r="A45" s="3">
         <v>44</v>
       </c>
-      <c r="B45" s="4"/>
+      <c r="B45" s="4" t="s">
+        <v>2114</v>
+      </c>
       <c r="C45" s="3" t="s">
         <v>133</v>
       </c>

</xml_diff>